<commit_message>
refactor: Update Excel download button text for products and materials, enhancing clarity in English and Korean translations
</commit_message>
<xml_diff>
--- a/frontend/public/product-excel.xlsx
+++ b/frontend/public/product-excel.xlsx
@@ -442,12 +442,12 @@
     <row r="1">
       <c r="A1" s="0" t="inlineStr">
         <is>
-          <t>품목명</t>
+          <t>제품명</t>
         </is>
       </c>
       <c r="B1" s="0" t="inlineStr">
         <is>
-          <t>품목코드</t>
+          <t>제품코드</t>
         </is>
       </c>
       <c r="C1" s="0" t="inlineStr">

</xml_diff>